<commit_message>
Deploying to gh-pages from  @ 50c295c7d9a4f7b2e53c5688044252fc9576fc8c 🚀
</commit_message>
<xml_diff>
--- a/en/downloads/data-excel/7.2.1.1.xlsx
+++ b/en/downloads/data-excel/7.2.1.1.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" showInkAnnotation="0" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9481050-65A3-4908-96E5-1DE125EA2290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -65,7 +66,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00_р_._-;\-* #,##0.00_р_._-;_-* &quot;-&quot;??_р_._-;_-@_-"/>
@@ -281,13 +282,12 @@
     <xf numFmtId="166" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -296,7 +296,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -305,75 +305,66 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Обычный 10" xfId="4"/>
-    <cellStyle name="Обычный 2" xfId="1"/>
-    <cellStyle name="Обычный 2 2" xfId="5"/>
-    <cellStyle name="Обычный 2 3" xfId="6"/>
-    <cellStyle name="Обычный 3" xfId="7"/>
-    <cellStyle name="Обычный 3 2" xfId="8"/>
-    <cellStyle name="Обычный 4" xfId="9"/>
-    <cellStyle name="Обычный 5" xfId="10"/>
-    <cellStyle name="Обычный 6" xfId="3"/>
-    <cellStyle name="Обычный 7" xfId="2"/>
-    <cellStyle name="Обычный 8" xfId="11"/>
-    <cellStyle name="Обычный 9" xfId="12"/>
-    <cellStyle name="Пояснение 2" xfId="13"/>
-    <cellStyle name="Процентный 2" xfId="14"/>
-    <cellStyle name="Процентный 3" xfId="15"/>
-    <cellStyle name="Стиль 1" xfId="16"/>
-    <cellStyle name="Финансовый 2" xfId="17"/>
-    <cellStyle name="Финансовый 3" xfId="18"/>
+    <cellStyle name="Обычный 10" xfId="4" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Обычный 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Обычный 2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Обычный 2 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Обычный 3" xfId="7" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Обычный 3 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Обычный 4" xfId="9" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Обычный 5" xfId="10" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Обычный 6" xfId="3" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Обычный 7" xfId="2" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Обычный 8" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Обычный 9" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Пояснение 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Процентный 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Процентный 3" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Стиль 1" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Финансовый 2" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Финансовый 3" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -389,9 +380,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -429,9 +420,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -466,7 +457,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -501,7 +492,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -674,255 +665,235 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="35.5703125" customWidth="1"/>
     <col min="4" max="20" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="12" customFormat="1" ht="42" customHeight="1">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:21" s="11" customFormat="1" ht="42" customHeight="1">
+      <c r="A1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:21">
+      <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
     </row>
-    <row r="3" spans="1:20" s="1" customFormat="1" ht="15.75" thickBot="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="4"/>
+    <row r="3" spans="1:21" ht="15.75" thickBot="1">
+      <c r="A3" s="1"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:21" ht="15.75" thickBot="1">
+      <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="17">
+      <c r="D4" s="16">
         <v>2007</v>
       </c>
-      <c r="E4" s="17">
+      <c r="E4" s="16">
         <v>2008</v>
       </c>
-      <c r="F4" s="17">
+      <c r="F4" s="16">
         <v>2009</v>
       </c>
-      <c r="G4" s="17">
+      <c r="G4" s="16">
         <v>2010</v>
       </c>
-      <c r="H4" s="17">
+      <c r="H4" s="16">
         <v>2011</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="16">
         <v>2012</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="16">
         <v>2013</v>
       </c>
-      <c r="K4" s="18">
+      <c r="K4" s="16">
         <v>2014</v>
       </c>
-      <c r="L4" s="17">
+      <c r="L4" s="16">
         <v>2015</v>
       </c>
-      <c r="M4" s="18">
+      <c r="M4" s="16">
         <v>2016</v>
       </c>
-      <c r="N4" s="18">
+      <c r="N4" s="16">
         <v>2017</v>
       </c>
-      <c r="O4" s="18">
+      <c r="O4" s="16">
         <v>2018</v>
       </c>
-      <c r="P4" s="18">
+      <c r="P4" s="16">
         <v>2019</v>
       </c>
-      <c r="Q4" s="18">
+      <c r="Q4" s="16">
         <v>2020</v>
       </c>
-      <c r="R4" s="18">
+      <c r="R4" s="16">
         <v>2021</v>
       </c>
-      <c r="S4" s="18">
+      <c r="S4" s="16">
         <v>2022</v>
       </c>
-      <c r="T4" s="18">
+      <c r="T4" s="16">
         <v>2023</v>
       </c>
+      <c r="U4" s="16">
+        <v>2024</v>
+      </c>
     </row>
-    <row r="5" spans="1:20" s="1" customFormat="1" ht="41.25" customHeight="1">
-      <c r="A5" s="19" t="s">
+    <row r="5" spans="1:21" ht="41.25" customHeight="1">
+      <c r="A5" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="12">
         <v>43.5</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="13">
         <v>36</v>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="12">
         <v>35.6</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="12">
         <v>38.700000000000003</v>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="13">
         <v>41</v>
       </c>
-      <c r="I5" s="13">
+      <c r="I5" s="12">
         <v>37.1</v>
       </c>
-      <c r="J5" s="13">
+      <c r="J5" s="12">
         <v>33.299999999999997</v>
       </c>
-      <c r="K5" s="13">
+      <c r="K5" s="12">
         <v>36.700000000000003</v>
       </c>
-      <c r="L5" s="13">
+      <c r="L5" s="12">
         <v>30.6</v>
       </c>
-      <c r="M5" s="13">
+      <c r="M5" s="12">
         <v>31.6</v>
       </c>
-      <c r="N5" s="13">
+      <c r="N5" s="12">
         <v>36.5</v>
       </c>
-      <c r="O5" s="13">
+      <c r="O5" s="12">
         <v>33.9</v>
       </c>
-      <c r="P5" s="14">
+      <c r="P5" s="13">
         <v>35.67</v>
       </c>
-      <c r="Q5" s="14">
+      <c r="Q5" s="13">
         <v>36.700000000000003</v>
       </c>
-      <c r="R5" s="13">
+      <c r="R5" s="12">
         <v>31.8</v>
       </c>
-      <c r="S5" s="13">
+      <c r="S5" s="12">
         <v>29.9</v>
       </c>
-      <c r="T5" s="13">
+      <c r="T5" s="12">
         <v>29.5</v>
       </c>
+      <c r="U5" s="13">
+        <v>28</v>
+      </c>
     </row>
-    <row r="6" spans="1:20" ht="28.5" customHeight="1" thickBot="1">
-      <c r="A6" s="22" t="s">
+    <row r="6" spans="1:21" ht="28.5" customHeight="1" thickBot="1">
+      <c r="A6" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="14">
         <v>14004.1</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="15">
         <v>10759.1</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="15">
         <v>10098</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="15">
         <v>11254.7</v>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="15">
         <v>14309.1</v>
       </c>
-      <c r="I6" s="16">
+      <c r="I6" s="15">
         <v>14179</v>
       </c>
-      <c r="J6" s="16">
+      <c r="J6" s="15">
         <v>13096.7</v>
       </c>
-      <c r="K6" s="16">
+      <c r="K6" s="15">
         <v>13297.6</v>
       </c>
-      <c r="L6" s="16">
+      <c r="L6" s="15">
         <v>11092.7</v>
       </c>
-      <c r="M6" s="15">
+      <c r="M6" s="14">
         <v>11497.8</v>
       </c>
-      <c r="N6" s="15">
+      <c r="N6" s="14">
         <v>14191.2</v>
       </c>
-      <c r="O6" s="15">
+      <c r="O6" s="14">
         <v>14318.3</v>
       </c>
-      <c r="P6" s="15">
+      <c r="P6" s="14">
         <v>13859.2</v>
       </c>
-      <c r="Q6" s="15">
+      <c r="Q6" s="14">
         <v>13979.2</v>
       </c>
-      <c r="R6" s="15">
+      <c r="R6" s="14">
         <v>12957.1</v>
       </c>
-      <c r="S6" s="15">
+      <c r="S6" s="14">
         <v>11928.6</v>
       </c>
-      <c r="T6" s="15">
+      <c r="T6" s="14">
         <v>12030.6</v>
       </c>
-    </row>
-    <row r="7" spans="1:20">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
+      <c r="U6" s="14">
+        <v>12935.8</v>
+      </c>
     </row>
   </sheetData>
   <dataConsolidate/>

</xml_diff>